<commit_message>
update dashboard + tarifs
</commit_message>
<xml_diff>
--- a/tarifs_colis_master.xlsx
+++ b/tarifs_colis_master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mathieujoostens/Documents/controle-transport-web/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BC9FDE4-B8ED-2149-AD14-1C012AFA3FE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83103209-A6C5-994D-9621-14E48B71A07A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6660" yWindow="4340" windowWidth="35100" windowHeight="15900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3300" yWindow="4340" windowWidth="35100" windowHeight="15900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tarifs" sheetId="2" r:id="rId1"/>
@@ -552,7 +552,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:T63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -636,7 +635,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -674,7 +673,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -712,7 +711,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -750,7 +749,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -788,7 +787,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -826,7 +825,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -864,7 +863,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -902,7 +901,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -940,7 +939,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -978,7 +977,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -1016,7 +1015,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -1054,7 +1053,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -1092,7 +1091,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>28</v>
       </c>
@@ -1130,7 +1129,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -1168,7 +1167,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>28</v>
       </c>
@@ -1206,7 +1205,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>28</v>
       </c>
@@ -1244,7 +1243,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>28</v>
       </c>
@@ -1282,7 +1281,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -1320,7 +1319,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>28</v>
       </c>
@@ -1358,7 +1357,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -1396,7 +1395,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>28</v>
       </c>
@@ -1434,7 +1433,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>28</v>
       </c>
@@ -1472,7 +1471,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -1510,7 +1509,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>28</v>
       </c>
@@ -1548,7 +1547,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="26" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>28</v>
       </c>
@@ -1586,7 +1585,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>28</v>
       </c>
@@ -1624,7 +1623,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="28" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>28</v>
       </c>
@@ -1662,7 +1661,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -1700,7 +1699,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -1738,7 +1737,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="31" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>28</v>
       </c>
@@ -1776,7 +1775,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="32" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>28</v>
       </c>
@@ -1814,7 +1813,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="33" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>28</v>
       </c>
@@ -1852,7 +1851,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>28</v>
       </c>
@@ -1890,7 +1889,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="35" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>28</v>
       </c>
@@ -1928,7 +1927,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="36" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>28</v>
       </c>
@@ -1966,7 +1965,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="37" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>28</v>
       </c>
@@ -2004,7 +2003,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="38" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>28</v>
       </c>
@@ -2042,7 +2041,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="39" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>28</v>
       </c>
@@ -2080,7 +2079,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="40" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>28</v>
       </c>
@@ -2118,7 +2117,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="41" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>28</v>
       </c>
@@ -2156,7 +2155,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="42" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>28</v>
       </c>
@@ -2194,7 +2193,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="43" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>28</v>
       </c>
@@ -2232,7 +2231,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="44" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>28</v>
       </c>
@@ -2270,7 +2269,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="45" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>28</v>
       </c>
@@ -2308,7 +2307,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="46" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>28</v>
       </c>
@@ -2346,7 +2345,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>28</v>
       </c>
@@ -2384,7 +2383,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="48" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>28</v>
       </c>
@@ -2422,7 +2421,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="49" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>28</v>
       </c>
@@ -2460,7 +2459,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="50" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>28</v>
       </c>
@@ -2498,7 +2497,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="51" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>28</v>
       </c>
@@ -2536,7 +2535,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="52" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>28</v>
       </c>
@@ -2574,7 +2573,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="53" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>28</v>
       </c>
@@ -3023,13 +3022,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T59" xr:uid="{00000000-0001-0000-0100-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="GLS"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:T59" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>